<commit_message>
Added in 2 datasets for the Feveriosis case study
Followed all instructions in the Adding data vignette.

Noting that in the Tableoftables.xlsx, the group and unique identifier formulas were broken (based on recent MS updates). I updated and then reviewed with main branch that they were the same.
</commit_message>
<xml_diff>
--- a/inst/extdata/tableoftables.xlsx
+++ b/inst/extdata/tableoftables.xlsx
@@ -1,22 +1,38 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10308"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alanahjansen/Documents/GitHub/appliedepidata/inst/extdata/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A071735-C90B-7A4F-9076-CE48082E0980}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="0"/>
+    <workbookView xWindow="-37800" yWindow="780" windowWidth="35640" windowHeight="18280" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr/>
+  <calcPr calcId="181029"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{D0CA8CA8-9F24-4464-BF8E-62219DCF47F9}"/>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="177">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="749" uniqueCount="184">
   <si>
     <t>name</t>
   </si>
@@ -87,7 +103,7 @@
     <t>subnational</t>
   </si>
   <si>
-    <t xml:space="preserve">acute jaundice syndrome</t>
+    <t>acute jaundice syndrome</t>
   </si>
   <si>
     <t>outbreak</t>
@@ -96,13 +112,13 @@
     <t>no</t>
   </si>
   <si>
-    <t xml:space="preserve">Linelist data from a real outbreak of Hepatitis E virus (HEV) infection which occurred in the town of Am Timan, Chad, between October 2016 and April 2017.</t>
+    <t>Linelist data from a real outbreak of Hepatitis E virus (HEV) infection which occurred in the town of Am Timan, Chad, between October 2016 and April 2017.</t>
   </si>
   <si>
     <t>sitrep_walkthroughs</t>
   </si>
   <si>
-    <t xml:space="preserve">CC by-NC-SA 4.0</t>
+    <t>CC by-NC-SA 4.0</t>
   </si>
   <si>
     <t>AJS_AmTiman_population</t>
@@ -111,7 +127,7 @@
     <t>population</t>
   </si>
   <si>
-    <t xml:space="preserve">Population data from an outbreak of Acute Jaundice Syndrome (AJS) in Chad 2016</t>
+    <t>Population data from an outbreak of Acute Jaundice Syndrome (AJS) in Chad 2016</t>
   </si>
   <si>
     <t>Blocksshape</t>
@@ -123,13 +139,13 @@
     <t>zip</t>
   </si>
   <si>
-    <t xml:space="preserve">Shapefile of housing blocks from an outbreak of Acute Jaundice Syndrome (AJS) in Chad 2016</t>
+    <t>Shapefile of housing blocks from an outbreak of Acute Jaundice Syndrome (AJS) in Chad 2016</t>
   </si>
   <si>
     <t>Quartiersshape</t>
   </si>
   <si>
-    <t xml:space="preserve">Shapefile of neighbourhoods (fr: quartiers) from an outbreak of Acute Jaundice Syndrome (AJS) in Chad 2016</t>
+    <t>Shapefile of neighbourhoods (fr: quartiers) from an outbreak of Acute Jaundice Syndrome (AJS) in Chad 2016</t>
   </si>
   <si>
     <t>mortality_survey_data</t>
@@ -147,7 +163,7 @@
     <t>yes</t>
   </si>
   <si>
-    <t xml:space="preserve">Fake data for a mortality survey</t>
+    <t>Fake data for a mortality survey</t>
   </si>
   <si>
     <t>gpl3</t>
@@ -159,7 +175,7 @@
     <t>dictionary</t>
   </si>
   <si>
-    <t xml:space="preserve">Fake data dictionary for a mortality survey</t>
+    <t>Fake data dictionary for a mortality survey</t>
   </si>
   <si>
     <t>franglais_AJS_AmTiman</t>
@@ -168,7 +184,7 @@
     <t>fr</t>
   </si>
   <si>
-    <t xml:space="preserve">quelque chose en francais - oui oui</t>
+    <t>quelque chose en francais - oui oui</t>
   </si>
   <si>
     <t>fulton_data</t>
@@ -180,7 +196,7 @@
     <t>covid-19</t>
   </si>
   <si>
-    <t xml:space="preserve">Jittered COVID-19 linelist data from Fulton County</t>
+    <t>Jittered COVID-19 linelist data from Fulton County</t>
   </si>
   <si>
     <t>case_studies</t>
@@ -210,7 +226,7 @@
     <t>mpox</t>
   </si>
   <si>
-    <t xml:space="preserve">Fictional mpox case linelist in five European countries</t>
+    <t>Fictional mpox case linelist in five European countries</t>
   </si>
   <si>
     <t>r_practical</t>
@@ -225,7 +241,7 @@
     <t>csv</t>
   </si>
   <si>
-    <t xml:space="preserve">Fictional cumulative mpox case counts in five European countries</t>
+    <t>Fictional cumulative mpox case counts in five European countries</t>
   </si>
   <si>
     <t>stegentira_data</t>
@@ -237,7 +253,7 @@
     <t>salmonella</t>
   </si>
   <si>
-    <t xml:space="preserve">Fictional linelist of salmonella outbreak in Stegen, Germany</t>
+    <t>Fictional linelist of salmonella outbreak in Stegen, Germany</t>
   </si>
   <si>
     <t>fluH7N9_China_2013</t>
@@ -252,7 +268,7 @@
     <t>influenza</t>
   </si>
   <si>
-    <t xml:space="preserve">Linelist data from an outbreak of influenza A H7N9 in China 2013.</t>
+    <t>Linelist data from an outbreak of influenza A H7N9 in China 2013.</t>
   </si>
   <si>
     <t>epirhandbook</t>
@@ -270,52 +286,52 @@
     <t>ebola</t>
   </si>
   <si>
-    <t xml:space="preserve">Fictional Ebola Virus Disease data simulating properties from the West African Ebola outbreak of 2014</t>
+    <t>Fictional Ebola Virus Disease data simulating properties from the West African Ebola outbreak of 2014</t>
   </si>
   <si>
     <t>linelist_cleaned_excel</t>
   </si>
   <si>
-    <t xml:space="preserve">Excel clean version of fictional Ebola Virus Disease data simulating properties from the West African Ebola outbreak of 2014</t>
+    <t>Excel clean version of fictional Ebola Virus Disease data simulating properties from the West African Ebola outbreak of 2014</t>
   </si>
   <si>
     <t>linelist_cleaned_rds</t>
   </si>
   <si>
-    <t xml:space="preserve">R-dataset clean version of fictional Ebola Virus Disease data simulating properties from the West African Ebola outbreak of 2014</t>
+    <t>R-dataset clean version of fictional Ebola Virus Disease data simulating properties from the West African Ebola outbreak of 2014</t>
   </si>
   <si>
     <t>hospital_linelists</t>
   </si>
   <si>
-    <t xml:space="preserve">Subset of excel clean version of fictional Ebola Virus Disease data simulating properties from the West African Ebola outbreak of 2014</t>
+    <t>Subset of excel clean version of fictional Ebola Virus Disease data simulating properties from the West African Ebola outbreak of 2014</t>
   </si>
   <si>
     <t>linelist_cleaned_with_adm3</t>
   </si>
   <si>
-    <t xml:space="preserve">Subset with additional spatial data of rds clean version of fictional Ebola Virus Disease data simulating properties from the West African Ebola outbreak of 2014</t>
+    <t>Subset with additional spatial data of rds clean version of fictional Ebola Virus Disease data simulating properties from the West African Ebola outbreak of 2014</t>
   </si>
   <si>
     <t>cleaning_dict</t>
   </si>
   <si>
-    <t xml:space="preserve">Short example cleaning dictionary for the raw linelist</t>
+    <t>Short example cleaning dictionary for the raw linelist</t>
   </si>
   <si>
     <t>sle_adm3</t>
   </si>
   <si>
-    <t xml:space="preserve">Shapefile at admin level  3 for Sierra Leone from Humanitarian Data Exchange</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CC by-IGO</t>
+    <t>Shapefile at admin level  3 for Sierra Leone from Humanitarian Data Exchange</t>
+  </si>
+  <si>
+    <t>CC by-IGO</t>
   </si>
   <si>
     <t>sle_admpop_adm3_2020</t>
   </si>
   <si>
-    <t xml:space="preserve">Population data at admin level 3 for Sierra Leone from Humanitarian Data Exchange</t>
+    <t>Population data at admin level 3 for Sierra Leone from Humanitarian Data Exchange</t>
   </si>
   <si>
     <t>epinow_res</t>
@@ -324,7 +340,7 @@
     <t>other</t>
   </si>
   <si>
-    <t xml:space="preserve">Outputs from {epinow2} based on fictional Ebola Virus Disease data simulating properties from the West African Ebola outbreak of 2014</t>
+    <t>Outputs from {epinow2} based on fictional Ebola Virus Disease data simulating properties from the West African Ebola outbreak of 2014</t>
   </si>
   <si>
     <t>epinow_res_small</t>
@@ -333,7 +349,7 @@
     <t>generation_time</t>
   </si>
   <si>
-    <t xml:space="preserve">Outputs from {epinow2} based on fictional Ebola Virus Disease data simulating properties from the West African Ebola outbreak of 2015</t>
+    <t>Outputs from {epinow2} based on fictional Ebola Virus Disease data simulating properties from the West African Ebola outbreak of 2015</t>
   </si>
   <si>
     <t>incubation_period</t>
@@ -342,10 +358,10 @@
     <t>cases_clean</t>
   </si>
   <si>
-    <t xml:space="preserve">contact tracing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fictional case data for a generic disease to demonstrate contact tracing</t>
+    <t>contact tracing</t>
+  </si>
+  <si>
+    <t>Fictional case data for a generic disease to demonstrate contact tracing</t>
   </si>
   <si>
     <t>contacts_clean</t>
@@ -366,7 +382,7 @@
     <t>malaria</t>
   </si>
   <si>
-    <t xml:space="preserve">Fictional counts of malaria cases from Mozambique</t>
+    <t>Fictional counts of malaria cases from Mozambique</t>
   </si>
   <si>
     <t>malaria_facility_count_data</t>
@@ -390,25 +406,25 @@
     <t>surveillance</t>
   </si>
   <si>
-    <t xml:space="preserve">Next generation sequencing data of Shigella surveillance samples from Belgium</t>
+    <t>Next generation sequencing data of Shigella surveillance samples from Belgium</t>
   </si>
   <si>
     <t>sample_data_Shigella_tree</t>
   </si>
   <si>
-    <t xml:space="preserve">Linelist data to accompany next generation sequencing data of Shigella surveillance samples from Belgium 2013-2019</t>
+    <t>Linelist data to accompany next generation sequencing data of Shigella surveillance samples from Belgium 2013-2019</t>
   </si>
   <si>
     <t>Shigella_subtree_2</t>
   </si>
   <si>
-    <t xml:space="preserve">Analysis output from next generation sequencing data of Shigella surveillance samples from Belgium</t>
+    <t>Analysis output from next generation sequencing data of Shigella surveillance samples from Belgium</t>
   </si>
   <si>
     <t>country_demographics</t>
   </si>
   <si>
-    <t xml:space="preserve">Fictional country demographic and mortality data to demonstrate standardisation</t>
+    <t>Fictional country demographic and mortality data to demonstrate standardisation</t>
   </si>
   <si>
     <t>country_demographics_2</t>
@@ -423,7 +439,7 @@
     <t>world_standard_population_by_sex</t>
   </si>
   <si>
-    <t xml:space="preserve">World “standard population” by sex</t>
+    <t>World “standard population” by sex</t>
   </si>
   <si>
     <t>OGL</t>
@@ -435,22 +451,22 @@
     <t>likert</t>
   </si>
   <si>
-    <t xml:space="preserve">Fictional likert data for demonstration purposes</t>
+    <t>Fictional likert data for demonstration purposes</t>
   </si>
   <si>
     <t>survey_data</t>
   </si>
   <si>
-    <t xml:space="preserve">Fictional data for a mortality survey</t>
+    <t>Fictional data for a mortality survey</t>
   </si>
   <si>
     <t>survey_dict</t>
   </si>
   <si>
-    <t xml:space="preserve">Fictional data dictionary for a mortality survey</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fictional population data for a mortality survey</t>
+    <t>Fictional data dictionary for a mortality survey</t>
+  </si>
+  <si>
+    <t>Fictional population data for a mortality survey</t>
   </si>
   <si>
     <t>campylobacter_germany</t>
@@ -459,7 +475,7 @@
     <t>campylobacter</t>
   </si>
   <si>
-    <t xml:space="preserve">Campylobacter surveillance data from Germany</t>
+    <t>Campylobacter surveillance data from Germany</t>
   </si>
   <si>
     <t>germany_weather</t>
@@ -468,7 +484,7 @@
     <t>weather</t>
   </si>
   <si>
-    <t xml:space="preserve">Weather data for Germany from 2001-2011</t>
+    <t>Weather data for Germany from 2001-2011</t>
   </si>
   <si>
     <t>multidisease_tests</t>
@@ -477,7 +493,7 @@
     <t>multidisease</t>
   </si>
   <si>
-    <t xml:space="preserve">Test results for notifiable diseases reported in Feveria in 2024</t>
+    <t>Test results for notifiable diseases reported in Feveria in 2024</t>
   </si>
   <si>
     <t>multidisease_surveillance</t>
@@ -486,7 +502,7 @@
     <t>multidisease_notifications</t>
   </si>
   <si>
-    <t xml:space="preserve">Notifiable disease surveillance data in Feveria in 2024</t>
+    <t>Notifiable disease surveillance data in Feveria in 2024</t>
   </si>
   <si>
     <t>multi_maladies_notifications</t>
@@ -519,61 +535,95 @@
     <t>cholera</t>
   </si>
   <si>
-    <t xml:space="preserve">Clean cholera surveillance data for Viraland, 25 May 2021</t>
-  </si>
-  <si>
-    <t xml:space="preserve">qmd, intror</t>
+    <t>Clean cholera surveillance data for Viraland, 25 May 2021</t>
+  </si>
+  <si>
+    <t>qmd, intror</t>
   </si>
   <si>
     <t>viraland_cholera_20210617_linelist</t>
   </si>
   <si>
-    <t xml:space="preserve">Clean cholera surveillance data for Viraland, 17 June 2021</t>
+    <t>Clean cholera surveillance data for Viraland, 17 June 2021</t>
   </si>
   <si>
     <t>viraland_cholera_20210721_linelist</t>
   </si>
   <si>
-    <t xml:space="preserve">Clean cholera surveillance data for Viraland, 21 July 2021</t>
+    <t>Clean cholera surveillance data for Viraland, 21 July 2021</t>
   </si>
   <si>
     <t>viraland_cholera_20210721_linelist_raw</t>
   </si>
   <si>
-    <t xml:space="preserve">Raw cholera surveillance data for Viraland, 21 July 2021</t>
+    <t>Raw cholera surveillance data for Viraland, 21 July 2021</t>
   </si>
   <si>
     <t>viraland_cholera_20210721_labs</t>
   </si>
   <si>
-    <t xml:space="preserve">Raw cholera lab data for Viraland, 21 July 2021</t>
+    <t>Raw cholera lab data for Viraland, 21 July 2021</t>
+  </si>
+  <si>
+    <t>feveriosis_main</t>
+  </si>
+  <si>
+    <t>Fake endemic vector-borne disease in Feveria 2025-26</t>
+  </si>
+  <si>
+    <t>feveriosis_surveillance</t>
+  </si>
+  <si>
+    <t>feveriosis_recent</t>
+  </si>
+  <si>
+    <t>Fake endemic vector-borne disease in Feveria 2025-27</t>
+  </si>
+  <si>
+    <t>CC by-NC-SA 4.1</t>
+  </si>
+  <si>
+    <t>feveriosis</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="4">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
-      <sz val="11.000000"/>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="11.000000"/>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11.500000"/>
+      <sz val="11.5"/>
       <name val="Calibri"/>
     </font>
     <font>
-      <sz val="11.000000"/>
+      <sz val="11"/>
       <name val="Times New Roman"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -586,31 +636,63 @@
   </fills>
   <borders count="1">
     <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
-    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf fontId="2" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+  <cellXfs count="6">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf fontId="3" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="3">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="2"/>
+          <bgColor indexed="2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -623,291 +705,8 @@
 </styleSheet>
 </file>
 
-<file path=xl/theme/theme.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
-  <a:themeElements>
-    <a:clrScheme name="Office">
-      <a:dk1>
-        <a:sysClr val="windowText" lastClr="000000"/>
-      </a:dk1>
-      <a:lt1>
-        <a:sysClr val="window" lastClr="FFFFFF"/>
-      </a:lt1>
-      <a:dk2>
-        <a:srgbClr val="1F497D"/>
-      </a:dk2>
-      <a:lt2>
-        <a:srgbClr val="EEECE1"/>
-      </a:lt2>
-      <a:accent1>
-        <a:srgbClr val="4F81BD"/>
-      </a:accent1>
-      <a:accent2>
-        <a:srgbClr val="C0504D"/>
-      </a:accent2>
-      <a:accent3>
-        <a:srgbClr val="9BBB59"/>
-      </a:accent3>
-      <a:accent4>
-        <a:srgbClr val="8064A2"/>
-      </a:accent4>
-      <a:accent5>
-        <a:srgbClr val="4BACC6"/>
-      </a:accent5>
-      <a:accent6>
-        <a:srgbClr val="F79646"/>
-      </a:accent6>
-      <a:hlink>
-        <a:srgbClr val="0000FF"/>
-      </a:hlink>
-      <a:folHlink>
-        <a:srgbClr val="800080"/>
-      </a:folHlink>
-    </a:clrScheme>
-    <a:fontScheme name="Office">
-      <a:majorFont>
-        <a:latin typeface="Cambria"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ ゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Angsana New"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-      </a:majorFont>
-      <a:minorFont>
-        <a:latin typeface="Calibri"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ 明朝"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Cordia New"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-      </a:minorFont>
-    </a:fontScheme>
-    <a:fmtScheme name="Office">
-      <a:fillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="50000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="35000">
-              <a:schemeClr val="phClr">
-                <a:tint val="37000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:tint val="15000"/>
-                <a:satMod val="350000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="16200000" scaled="1"/>
-        </a:gradFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:shade val="51000"/>
-                <a:satMod val="130000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="80000">
-              <a:schemeClr val="phClr">
-                <a:shade val="93000"/>
-                <a:satMod val="130000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="94000"/>
-                <a:satMod val="135000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="16200000" scaled="0"/>
-        </a:gradFill>
-      </a:fillStyleLst>
-      <a:lnStyleLst>
-        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr">
-              <a:shade val="95000"/>
-              <a:satMod val="105000"/>
-            </a:schemeClr>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </a:lnStyleLst>
-      <a:effectStyleLst>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="38000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="35000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="35000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-          <a:scene3d>
-            <a:camera prst="orthographicFront">
-              <a:rot lat="0" lon="0" rev="0"/>
-            </a:camera>
-            <a:lightRig rig="threePt" dir="t">
-              <a:rot lat="0" lon="0" rev="1200000"/>
-            </a:lightRig>
-          </a:scene3d>
-          <a:sp3d>
-            <a:bevelT w="63500" h="25400"/>
-          </a:sp3d>
-        </a:effectStyle>
-      </a:effectStyleLst>
-      <a:bgFillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="40000"/>
-                <a:satMod val="350000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="40000">
-              <a:schemeClr val="phClr">
-                <a:tint val="45000"/>
-                <a:shade val="99000"/>
-                <a:satMod val="350000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="20000"/>
-                <a:satMod val="255000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
-          </a:path>
-        </a:gradFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="80000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="30000"/>
-                <a:satMod val="200000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
-          </a:path>
-        </a:gradFill>
-      </a:bgFillStyleLst>
-    </a:fmtScheme>
-  </a:themeElements>
-  <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
-</a:theme>
-</file>
-
-<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:p="http://schemas.openxmlformats.org/presentationml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="New Office">
       <a:dk1>
@@ -1110,29 +909,31 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
-  <sheetFormatPr defaultColWidth="8.83984375" defaultRowHeight="14.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:Q62"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="44.26171875"/>
-    <col customWidth="1" min="2" max="2" width="10.3125"/>
+    <col min="1" max="1" width="44.33203125" customWidth="1"/>
+    <col min="2" max="2" width="10.33203125" customWidth="1"/>
     <col min="3" max="3" width="9"/>
-    <col bestFit="1" customWidth="1" min="4" max="5" width="12.15625"/>
-    <col bestFit="1" min="8" max="8" width="10.68359375"/>
-    <col bestFit="1" min="9" max="9" width="22.47265625"/>
-    <col customWidth="1" min="10" max="11" width="11.15625"/>
-    <col customWidth="1" min="12" max="12" width="5.68359375"/>
-    <col bestFit="1" min="13" max="13" width="10.47265625"/>
-    <col bestFit="1" min="14" max="14" width="18.15625"/>
-    <col bestFit="1" min="15" max="15" width="14.3125"/>
-    <col bestFit="1" min="16" max="16" width="39.68359375"/>
-    <col bestFit="1" min="17" max="17" width="67.47265625"/>
+    <col min="4" max="5" width="12.1640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.6640625" bestFit="1"/>
+    <col min="9" max="9" width="22.5" bestFit="1"/>
+    <col min="10" max="11" width="11.1640625" customWidth="1"/>
+    <col min="12" max="12" width="5.6640625" customWidth="1"/>
+    <col min="13" max="13" width="10.5" bestFit="1"/>
+    <col min="14" max="14" width="18.1640625" bestFit="1"/>
+    <col min="15" max="15" width="14.33203125" bestFit="1"/>
+    <col min="16" max="16" width="39.6640625" bestFit="1"/>
+    <col min="17" max="17" width="67.5" bestFit="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15.550000000000001" customHeight="1">
+    <row r="1" spans="1:17" ht="15.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1185,7 +986,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>17</v>
       </c>
@@ -1232,15 +1033,15 @@
         <v>28</v>
       </c>
       <c r="P2" t="str">
-        <f t="shared" ref="P2:P9" si="0">_xlfn.CONCAT(SUBSTITUTE(I2," ",""),"_",J2,"_",G2,"_",L2)</f>
+        <f>CONCATENATE(SUBSTITUTE(I2," ",""),"_",J2,"_",G2,"_",L2)</f>
         <v>acutejaundicesyndrome_outbreak_tcd_2016</v>
       </c>
       <c r="Q2" t="str">
-        <f t="shared" ref="Q2:Q33" si="1">_xlfn.CONCAT(P2,"_",B2,"_",D2,"_",E2)</f>
+        <f>CONCATENATE(P2,"_",B2,"_",D2,"_",E2)</f>
         <v>acutejaundicesyndrome_outbreak_tcd_2016_linelist_1_1</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>29</v>
       </c>
@@ -1287,15 +1088,15 @@
         <v>28</v>
       </c>
       <c r="P3" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="P3:P62" si="0">CONCATENATE(SUBSTITUTE(I3," ",""),"_",J3,"_",G3,"_",L3)</f>
         <v>acutejaundicesyndrome_outbreak_tcd_2016</v>
       </c>
       <c r="Q3" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" ref="Q3:Q62" si="1">CONCATENATE(P3,"_",B3,"_",D3,"_",E3)</f>
         <v>acutejaundicesyndrome_outbreak_tcd_2016_population_1_1</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>32</v>
       </c>
@@ -1350,7 +1151,7 @@
         <v>acutejaundicesyndrome_outbreak_tcd_2016_shape_1_1</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>36</v>
       </c>
@@ -1405,7 +1206,7 @@
         <v>acutejaundicesyndrome_outbreak_tcd_2016_shape_2_1</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>38</v>
       </c>
@@ -1460,7 +1261,7 @@
         <v>mortality_survey_zzz_2021_survey_1_1</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>45</v>
       </c>
@@ -1515,7 +1316,7 @@
         <v>mortality_survey_zzz_2021_dictionary_1_1</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>48</v>
       </c>
@@ -1570,7 +1371,7 @@
         <v>acutejaundicesyndrome_outbreak_tcd_2016_linelist_1_1</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>51</v>
       </c>
@@ -1625,7 +1426,7 @@
         <v>covid-19_outbreak_usa_2020_linelist_1_1</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>56</v>
       </c>
@@ -1672,7 +1473,7 @@
         <v>28</v>
       </c>
       <c r="P10" t="str">
-        <f t="shared" ref="P10:P60" si="2">_xlfn.CONCAT(SUBSTITUTE(I10," ",""),"_",J10,"_",G10,"_",L10)</f>
+        <f t="shared" si="0"/>
         <v>covid-19_outbreak_usa_2020</v>
       </c>
       <c r="Q10" t="str">
@@ -1680,7 +1481,7 @@
         <v>covid-19_outbreak_usa_2020_linelist_1_2</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>58</v>
       </c>
@@ -1727,7 +1528,7 @@
         <v>28</v>
       </c>
       <c r="P11" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>covid-19_outbreak_usa_2020</v>
       </c>
       <c r="Q11" t="str">
@@ -1735,7 +1536,7 @@
         <v>covid-19_outbreak_usa_2020_population_1_1</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>60</v>
       </c>
@@ -1782,7 +1583,7 @@
         <v>28</v>
       </c>
       <c r="P12" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>mpox_outbreak_eue_2022</v>
       </c>
       <c r="Q12" t="str">
@@ -1790,7 +1591,7 @@
         <v>mpox_outbreak_eue_2022_linelist_1_1</v>
       </c>
     </row>
-    <row r="13">
+    <row r="13" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>66</v>
       </c>
@@ -1837,7 +1638,7 @@
         <v>28</v>
       </c>
       <c r="P13" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>mpox_outbreak_eue_2022</v>
       </c>
       <c r="Q13" t="str">
@@ -1845,7 +1646,7 @@
         <v>mpox_outbreak_eue_2022_aggregate_1_1</v>
       </c>
     </row>
-    <row r="14">
+    <row r="14" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>70</v>
       </c>
@@ -1892,7 +1693,7 @@
         <v>28</v>
       </c>
       <c r="P14" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>salmonella_outbreak_deu_1998</v>
       </c>
       <c r="Q14" t="str">
@@ -1900,7 +1701,7 @@
         <v>salmonella_outbreak_deu_1998_linelist_1_1</v>
       </c>
     </row>
-    <row r="15">
+    <row r="15" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>74</v>
       </c>
@@ -1947,7 +1748,7 @@
         <v>80</v>
       </c>
       <c r="P15" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>influenza_outbreak_chn_2013</v>
       </c>
       <c r="Q15" t="str">
@@ -1955,7 +1756,7 @@
         <v>influenza_outbreak_chn_2013_linelist_1_1</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>81</v>
       </c>
@@ -2002,7 +1803,7 @@
         <v>80</v>
       </c>
       <c r="P16" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>ebola_outbreak_sle_2014</v>
       </c>
       <c r="Q16" t="str">
@@ -2010,7 +1811,7 @@
         <v>ebola_outbreak_sle_2014_linelist_1_1</v>
       </c>
     </row>
-    <row r="17">
+    <row r="17" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>85</v>
       </c>
@@ -2057,7 +1858,7 @@
         <v>80</v>
       </c>
       <c r="P17" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>ebola_outbreak_sle_2014</v>
       </c>
       <c r="Q17" t="str">
@@ -2065,7 +1866,7 @@
         <v>ebola_outbreak_sle_2014_linelist_1_2</v>
       </c>
     </row>
-    <row r="18">
+    <row r="18" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>87</v>
       </c>
@@ -2112,7 +1913,7 @@
         <v>80</v>
       </c>
       <c r="P18" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>ebola_outbreak_sle_2014</v>
       </c>
       <c r="Q18" t="str">
@@ -2120,7 +1921,7 @@
         <v>ebola_outbreak_sle_2014_linelist_1_3</v>
       </c>
     </row>
-    <row r="19">
+    <row r="19" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>89</v>
       </c>
@@ -2167,7 +1968,7 @@
         <v>80</v>
       </c>
       <c r="P19" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>ebola_outbreak_sle_2014</v>
       </c>
       <c r="Q19" t="str">
@@ -2175,7 +1976,7 @@
         <v>ebola_outbreak_sle_2014_linelist_1_4</v>
       </c>
     </row>
-    <row r="20">
+    <row r="20" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>91</v>
       </c>
@@ -2222,7 +2023,7 @@
         <v>80</v>
       </c>
       <c r="P20" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>ebola_outbreak_sle_2014</v>
       </c>
       <c r="Q20" t="str">
@@ -2230,7 +2031,7 @@
         <v>ebola_outbreak_sle_2014_linelist_1_5</v>
       </c>
     </row>
-    <row r="21">
+    <row r="21" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>93</v>
       </c>
@@ -2277,7 +2078,7 @@
         <v>80</v>
       </c>
       <c r="P21" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>ebola_outbreak_sle_2014</v>
       </c>
       <c r="Q21" t="str">
@@ -2285,7 +2086,7 @@
         <v>ebola_outbreak_sle_2014_dictionary_1_1</v>
       </c>
     </row>
-    <row r="22">
+    <row r="22" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>95</v>
       </c>
@@ -2332,7 +2133,7 @@
         <v>97</v>
       </c>
       <c r="P22" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>ebola_outbreak_sle_2014</v>
       </c>
       <c r="Q22" t="str">
@@ -2340,7 +2141,7 @@
         <v>ebola_outbreak_sle_2014_shape_1_1</v>
       </c>
     </row>
-    <row r="23">
+    <row r="23" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>98</v>
       </c>
@@ -2387,7 +2188,7 @@
         <v>97</v>
       </c>
       <c r="P23" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>ebola_outbreak_sle_2020</v>
       </c>
       <c r="Q23" t="str">
@@ -2395,7 +2196,7 @@
         <v>ebola_outbreak_sle_2020_population_1_1</v>
       </c>
     </row>
-    <row r="24" ht="15.75">
+    <row r="24" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A24" s="2" t="s">
         <v>100</v>
       </c>
@@ -2442,7 +2243,7 @@
         <v>80</v>
       </c>
       <c r="P24" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>ebola_outbreak_sle_2014</v>
       </c>
       <c r="Q24" t="str">
@@ -2450,7 +2251,7 @@
         <v>ebola_outbreak_sle_2014_other_1_1</v>
       </c>
     </row>
-    <row r="25" ht="15.75">
+    <row r="25" spans="1:17" ht="16" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
         <v>103</v>
       </c>
@@ -2497,7 +2298,7 @@
         <v>80</v>
       </c>
       <c r="P25" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>ebola_outbreak_sle_2014</v>
       </c>
       <c r="Q25" t="str">
@@ -2505,7 +2306,7 @@
         <v>ebola_outbreak_sle_2014_other_2_1</v>
       </c>
     </row>
-    <row r="26">
+    <row r="26" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>104</v>
       </c>
@@ -2552,7 +2353,7 @@
         <v>80</v>
       </c>
       <c r="P26" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>ebola_outbreak_sle_2014</v>
       </c>
       <c r="Q26" t="str">
@@ -2560,7 +2361,7 @@
         <v>ebola_outbreak_sle_2014_other_3_1</v>
       </c>
     </row>
-    <row r="27">
+    <row r="27" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>106</v>
       </c>
@@ -2607,7 +2408,7 @@
         <v>80</v>
       </c>
       <c r="P27" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>ebola_outbreak_sle_2014</v>
       </c>
       <c r="Q27" t="str">
@@ -2615,7 +2416,7 @@
         <v>ebola_outbreak_sle_2014_other_4_1</v>
       </c>
     </row>
-    <row r="28">
+    <row r="28" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>107</v>
       </c>
@@ -2662,7 +2463,7 @@
         <v>44</v>
       </c>
       <c r="P28" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>contacttracing_outbreak_zzz_2020</v>
       </c>
       <c r="Q28" t="str">
@@ -2670,7 +2471,7 @@
         <v>contacttracing_outbreak_zzz_2020_linelist_1_1</v>
       </c>
     </row>
-    <row r="29">
+    <row r="29" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>110</v>
       </c>
@@ -2717,7 +2518,7 @@
         <v>44</v>
       </c>
       <c r="P29" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>contacttracing_outbreak_zzz_2020</v>
       </c>
       <c r="Q29" t="str">
@@ -2725,7 +2526,7 @@
         <v>contacttracing_outbreak_zzz_2020_linelist_2_1</v>
       </c>
     </row>
-    <row r="30">
+    <row r="30" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>111</v>
       </c>
@@ -2772,7 +2573,7 @@
         <v>44</v>
       </c>
       <c r="P30" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>contacttracing_outbreak_zzz_2020</v>
       </c>
       <c r="Q30" t="str">
@@ -2780,7 +2581,7 @@
         <v>contacttracing_outbreak_zzz_2020_linelist_3_1</v>
       </c>
     </row>
-    <row r="31">
+    <row r="31" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>112</v>
       </c>
@@ -2827,7 +2628,7 @@
         <v>44</v>
       </c>
       <c r="P31" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>contacttracing_outbreak_zzz_2020</v>
       </c>
       <c r="Q31" t="str">
@@ -2835,7 +2636,7 @@
         <v>contacttracing_outbreak_zzz_2020_linelist_4_1</v>
       </c>
     </row>
-    <row r="32">
+    <row r="32" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>113</v>
       </c>
@@ -2882,7 +2683,7 @@
         <v>28</v>
       </c>
       <c r="P32" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>malaria_outbreak_moz_2019</v>
       </c>
       <c r="Q32" t="str">
@@ -2890,7 +2691,7 @@
         <v>malaria_outbreak_moz_2019_aggregate_1_1</v>
       </c>
     </row>
-    <row r="33">
+    <row r="33" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>117</v>
       </c>
@@ -2937,7 +2738,7 @@
         <v>28</v>
       </c>
       <c r="P33" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>malaria_outbreak_moz_2019</v>
       </c>
       <c r="Q33" t="str">
@@ -2945,7 +2746,7 @@
         <v>malaria_outbreak_moz_2019_aggregate_1_2</v>
       </c>
     </row>
-    <row r="34">
+    <row r="34" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>118</v>
       </c>
@@ -2992,15 +2793,15 @@
         <v>28</v>
       </c>
       <c r="P34" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>shigella_surveillance_bel_2013</v>
       </c>
       <c r="Q34" t="str">
-        <f t="shared" ref="Q34:Q65" si="3">_xlfn.CONCAT(P34,"_",B34,"_",D34,"_",E34)</f>
+        <f t="shared" si="1"/>
         <v>shigella_surveillance_bel_2013_sequencing_1_1</v>
       </c>
     </row>
-    <row r="35" ht="15.550000000000001" customHeight="1">
+    <row r="35" spans="1:17" ht="15.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>125</v>
       </c>
@@ -3047,15 +2848,15 @@
         <v>28</v>
       </c>
       <c r="P35" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>shigella_surveillance_bel_2013</v>
       </c>
       <c r="Q35" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>shigella_surveillance_bel_2013_linelist_1_1</v>
       </c>
     </row>
-    <row r="36">
+    <row r="36" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>127</v>
       </c>
@@ -3102,15 +2903,15 @@
         <v>28</v>
       </c>
       <c r="P36" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>shigella_surveillance_bel_2013</v>
       </c>
       <c r="Q36" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>shigella_surveillance_bel_2013_sequencing_1_2</v>
       </c>
     </row>
-    <row r="37">
+    <row r="37" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>129</v>
       </c>
@@ -3157,15 +2958,15 @@
         <v>28</v>
       </c>
       <c r="P37" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>mortality_surveillance_zzz_2020</v>
       </c>
       <c r="Q37" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>mortality_surveillance_zzz_2020_aggregate_1_1</v>
       </c>
     </row>
-    <row r="38">
+    <row r="38" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>131</v>
       </c>
@@ -3212,15 +3013,15 @@
         <v>28</v>
       </c>
       <c r="P38" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>mortality_surveillance_zzz_2020</v>
       </c>
       <c r="Q38" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>mortality_surveillance_zzz_2020_aggregate_2_1</v>
       </c>
     </row>
-    <row r="39">
+    <row r="39" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>132</v>
       </c>
@@ -3267,15 +3068,15 @@
         <v>28</v>
       </c>
       <c r="P39" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>mortality_surveillance_zzz_2020</v>
       </c>
       <c r="Q39" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>mortality_surveillance_zzz_2020_aggregate_3_1</v>
       </c>
     </row>
-    <row r="40">
+    <row r="40" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>133</v>
       </c>
@@ -3322,15 +3123,15 @@
         <v>28</v>
       </c>
       <c r="P40" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>mortality_surveillance_zzz_2020</v>
       </c>
       <c r="Q40" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>mortality_surveillance_zzz_2020_aggregate_4_1</v>
       </c>
     </row>
-    <row r="41">
+    <row r="41" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>134</v>
       </c>
@@ -3377,15 +3178,15 @@
         <v>136</v>
       </c>
       <c r="P41" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>mortality_surveillance_zzz_2020</v>
       </c>
       <c r="Q41" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>mortality_surveillance_zzz_2020_aggregate_5_1</v>
       </c>
     </row>
-    <row r="42">
+    <row r="42" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>137</v>
       </c>
@@ -3432,15 +3233,15 @@
         <v>28</v>
       </c>
       <c r="P42" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>likert_other_zzz_2020</v>
       </c>
       <c r="Q42" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>likert_other_zzz_2020_aggregate_1_1</v>
       </c>
     </row>
-    <row r="43">
+    <row r="43" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>140</v>
       </c>
@@ -3487,15 +3288,15 @@
         <v>44</v>
       </c>
       <c r="P43" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>mortality_survey_zzz_2021</v>
       </c>
       <c r="Q43" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>mortality_survey_zzz_2021_survey_2_1</v>
       </c>
     </row>
-    <row r="44">
+    <row r="44" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>142</v>
       </c>
@@ -3542,15 +3343,15 @@
         <v>44</v>
       </c>
       <c r="P44" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>mortality_survey_zzz_2021</v>
       </c>
       <c r="Q44" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>mortality_survey_zzz_2021_dictionary_2_1</v>
       </c>
     </row>
-    <row r="45">
+    <row r="45" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>30</v>
       </c>
@@ -3597,15 +3398,15 @@
         <v>44</v>
       </c>
       <c r="P45" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>mortality_survey_zzz_2021</v>
       </c>
       <c r="Q45" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>mortality_survey_zzz_2021_population_1_1</v>
       </c>
     </row>
-    <row r="46">
+    <row r="46" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>145</v>
       </c>
@@ -3652,15 +3453,15 @@
         <v>44</v>
       </c>
       <c r="P46" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>campylobacter_surveillance_deu_2001</v>
       </c>
       <c r="Q46" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>campylobacter_surveillance_deu_2001_linelist_1_1</v>
       </c>
     </row>
-    <row r="47">
+    <row r="47" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>148</v>
       </c>
@@ -3707,15 +3508,15 @@
         <v>44</v>
       </c>
       <c r="P47" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>weather_other_deu_2001</v>
       </c>
       <c r="Q47" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>weather_other_deu_2001_aggregate_1_1</v>
       </c>
     </row>
-    <row r="48">
+    <row r="48" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>151</v>
       </c>
@@ -3762,15 +3563,15 @@
         <v>28</v>
       </c>
       <c r="P48" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>multidisease_surveillance_zzz_2024</v>
       </c>
       <c r="Q48" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>multidisease_surveillance_zzz_2024_linelist_1_1</v>
       </c>
     </row>
-    <row r="49">
+    <row r="49" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>155</v>
       </c>
@@ -3817,15 +3618,15 @@
         <v>28</v>
       </c>
       <c r="P49" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>multidisease_surveillance_zzz_2024</v>
       </c>
       <c r="Q49" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>multidisease_surveillance_zzz_2024_linelist_2_1</v>
       </c>
     </row>
-    <row r="50">
+    <row r="50" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>157</v>
       </c>
@@ -3872,15 +3673,15 @@
         <v>28</v>
       </c>
       <c r="P50" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>multidisease_surveillance_zzz_2024</v>
       </c>
       <c r="Q50" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>multidisease_surveillance_zzz_2024_linelist_2_1</v>
       </c>
     </row>
-    <row r="51">
+    <row r="51" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>158</v>
       </c>
@@ -3927,15 +3728,15 @@
         <v>28</v>
       </c>
       <c r="P51" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>multidisease_surveillance_zzz_2024</v>
       </c>
       <c r="Q51" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>multidisease_surveillance_zzz_2024_linelist_1_1</v>
       </c>
     </row>
-    <row r="52">
+    <row r="52" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>159</v>
       </c>
@@ -3982,15 +3783,15 @@
         <v>28</v>
       </c>
       <c r="P52" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>multidisease_surveillance_zzz_2024</v>
       </c>
       <c r="Q52" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>multidisease_surveillance_zzz_2024_linelist_2_1</v>
       </c>
     </row>
-    <row r="53">
+    <row r="53" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>161</v>
       </c>
@@ -4037,15 +3838,15 @@
         <v>28</v>
       </c>
       <c r="P53" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>multidisease_surveillance_zzz_2024</v>
       </c>
       <c r="Q53" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>multidisease_surveillance_zzz_2024_linelist_1_1</v>
       </c>
     </row>
-    <row r="54">
+    <row r="54" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>162</v>
       </c>
@@ -4092,15 +3893,15 @@
         <v>28</v>
       </c>
       <c r="P54" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>multidisease_surveillance_zzz_2024</v>
       </c>
       <c r="Q54" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>multidisease_surveillance_zzz_2024_linelist_2_1</v>
       </c>
     </row>
-    <row r="55">
+    <row r="55" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>164</v>
       </c>
@@ -4147,15 +3948,15 @@
         <v>28</v>
       </c>
       <c r="P55" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>multidisease_surveillance_zzz_2024</v>
       </c>
       <c r="Q55" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>multidisease_surveillance_zzz_2024_linelist_1_1</v>
       </c>
     </row>
-    <row r="56">
+    <row r="56" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>165</v>
       </c>
@@ -4202,15 +4003,15 @@
         <v>28</v>
       </c>
       <c r="P56" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>cholera_surveillance_zzz_2021</v>
       </c>
       <c r="Q56" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>cholera_surveillance_zzz_2021_linelist_1_3</v>
       </c>
     </row>
-    <row r="57">
+    <row r="57" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>169</v>
       </c>
@@ -4250,22 +4051,22 @@
       <c r="M57" t="s">
         <v>170</v>
       </c>
-      <c r="N57" s="4" t="s">
+      <c r="N57" t="s">
         <v>168</v>
       </c>
       <c r="O57" t="s">
         <v>28</v>
       </c>
       <c r="P57" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>cholera_surveillance_zzz_2021</v>
       </c>
       <c r="Q57" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>cholera_surveillance_zzz_2021_linelist_1_4</v>
       </c>
     </row>
-    <row r="58">
+    <row r="58" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>171</v>
       </c>
@@ -4305,22 +4106,22 @@
       <c r="M58" t="s">
         <v>172</v>
       </c>
-      <c r="N58" s="4" t="s">
+      <c r="N58" t="s">
         <v>168</v>
       </c>
       <c r="O58" t="s">
         <v>28</v>
       </c>
       <c r="P58" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>cholera_surveillance_zzz_2021</v>
       </c>
       <c r="Q58" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>cholera_surveillance_zzz_2021_linelist_1_1</v>
       </c>
     </row>
-    <row r="59">
+    <row r="59" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>173</v>
       </c>
@@ -4360,22 +4161,22 @@
       <c r="M59" t="s">
         <v>174</v>
       </c>
-      <c r="N59" s="4" t="s">
+      <c r="N59" t="s">
         <v>168</v>
       </c>
       <c r="O59" t="s">
         <v>28</v>
       </c>
       <c r="P59" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>cholera_surveillance_zzz_2021</v>
       </c>
       <c r="Q59" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>cholera_surveillance_zzz_2021_linelist_1_2</v>
       </c>
     </row>
-    <row r="60">
+    <row r="60" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
         <v>175</v>
       </c>
@@ -4415,77 +4216,145 @@
       <c r="M60" t="s">
         <v>176</v>
       </c>
-      <c r="N60" s="4" t="s">
+      <c r="N60" t="s">
         <v>168</v>
       </c>
       <c r="O60" t="s">
         <v>28</v>
       </c>
       <c r="P60" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>cholera_surveillance_zzz_2021</v>
       </c>
       <c r="Q60" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>cholera_surveillance_zzz_2021_linelist_1_5</v>
       </c>
     </row>
+    <row r="61" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A61" s="5" t="s">
+        <v>177</v>
+      </c>
+      <c r="B61" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C61" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D61">
+        <v>1</v>
+      </c>
+      <c r="E61">
+        <v>1</v>
+      </c>
+      <c r="F61" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="G61" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="H61" t="s">
+        <v>76</v>
+      </c>
+      <c r="I61" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="J61" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="K61" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="L61">
+        <v>2025</v>
+      </c>
+      <c r="M61" s="4" t="s">
+        <v>178</v>
+      </c>
+      <c r="N61" s="4" t="s">
+        <v>179</v>
+      </c>
+      <c r="O61" t="s">
+        <v>28</v>
+      </c>
+      <c r="P61" t="str">
+        <f t="shared" si="0"/>
+        <v>feveriosis_surveillance_zzz_2025</v>
+      </c>
+      <c r="Q61" t="str">
+        <f t="shared" si="1"/>
+        <v>feveriosis_surveillance_zzz_2025_linelist_1_1</v>
+      </c>
+    </row>
+    <row r="62" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A62" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="B62" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C62" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="D62">
+        <v>2</v>
+      </c>
+      <c r="E62">
+        <v>1</v>
+      </c>
+      <c r="F62" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="G62" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="H62" t="s">
+        <v>76</v>
+      </c>
+      <c r="I62" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="J62" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="K62" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="L62">
+        <v>2025</v>
+      </c>
+      <c r="M62" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="N62" s="4" t="s">
+        <v>179</v>
+      </c>
+      <c r="O62" t="s">
+        <v>182</v>
+      </c>
+      <c r="P62" t="str">
+        <f t="shared" si="0"/>
+        <v>feveriosis_surveillance_zzz_2025</v>
+      </c>
+      <c r="Q62" t="str">
+        <f t="shared" si="1"/>
+        <v>feveriosis_surveillance_zzz_2025_linelist_2_1</v>
+      </c>
+    </row>
   </sheetData>
-  <printOptions headings="0" gridLines="0"/>
-  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
-  <headerFooter/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
-      <x14:conditionalFormattings>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="duplicateValues" priority="3" id="{00DA006C-00CF-44EB-B19D-0047002000B9}">
-            <x14:dxf>
-              <font>
-                <color rgb="FF9C0006"/>
-              </font>
-              <fill>
-                <patternFill patternType="solid">
-                  <fgColor rgb="FFFFC7CE"/>
-                  <bgColor rgb="FFFFC7CE"/>
-                </patternFill>
-              </fill>
-            </x14:dxf>
-          </x14:cfRule>
-          <xm:sqref>A1:A53 A56:A1048576</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="duplicateValues" priority="4" id="{002A0088-0095-4F59-A247-0052005900F4}">
-            <x14:dxf>
-              <font>
-                <color rgb="FF9C0006"/>
-              </font>
-              <fill>
-                <patternFill patternType="solid">
-                  <fgColor rgb="FFFFC7CE"/>
-                  <bgColor rgb="FFFFC7CE"/>
-                </patternFill>
-              </fill>
-            </x14:dxf>
-          </x14:cfRule>
-          <xm:sqref>A25</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="expression" priority="1" id="{00F0009D-0044-498A-8203-005F00AF00AA}">
-            <xm:f>AND(LEN(G2)&lt;&gt;3,LEN(G2)&lt;&gt;0)</xm:f>
-            <x14:dxf>
-              <fill>
-                <patternFill patternType="solid">
-                  <fgColor indexed="2"/>
-                  <bgColor indexed="2"/>
-                </patternFill>
-              </fill>
-            </x14:dxf>
-          </x14:cfRule>
-          <xm:sqref>G2:G300 K56:K60</xm:sqref>
-        </x14:conditionalFormatting>
-      </x14:conditionalFormattings>
-    </ext>
-  </extLst>
+  <phoneticPr fontId="5" type="noConversion"/>
+  <conditionalFormatting sqref="A1:A53 A56:A1048576">
+    <cfRule type="duplicateValues" dxfId="2" priority="3"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A25">
+    <cfRule type="duplicateValues" dxfId="1" priority="4"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K56:K62 G2:G300">
+    <cfRule type="expression" dxfId="0" priority="1">
+      <formula>AND(LEN(G2)&lt;&gt;3,LEN(G2)&lt;&gt;0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Added in updated datasets
Steps included:
- removing original datasets
- adding new datasets and rebuilding
- updating tableoftables (data_version = 2)
- re-running feveriosis_main.R and feveriosis_recent.R to save both datasets as .rda files
- updating documentation with proper version numbers and dataset info and re-running devtools::document()
</commit_message>
<xml_diff>
--- a/inst/extdata/tableoftables.xlsx
+++ b/inst/extdata/tableoftables.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alanahjansen/Documents/GitHub/appliedepidata/inst/extdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF635EF5-22EF-7041-BBB8-276C994C7A7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63E96078-6B29-F744-B65D-81FD1DAC6F78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-37800" yWindow="780" windowWidth="35640" windowHeight="18280" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-34960" yWindow="1920" windowWidth="35640" windowHeight="18280" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -4244,7 +4244,7 @@
         <v>1</v>
       </c>
       <c r="E61">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F61" s="4" t="s">
         <v>20</v>
@@ -4282,7 +4282,7 @@
       </c>
       <c r="Q61" t="str">
         <f t="shared" si="1"/>
-        <v>feveriosis_surveillance_zzz_2025_linelist_1_1</v>
+        <v>feveriosis_surveillance_zzz_2025_linelist_1_2</v>
       </c>
     </row>
     <row r="62" spans="1:17" x14ac:dyDescent="0.2">
@@ -4299,7 +4299,7 @@
         <v>2</v>
       </c>
       <c r="E62">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F62" s="4" t="s">
         <v>20</v>
@@ -4337,7 +4337,7 @@
       </c>
       <c r="Q62" t="str">
         <f t="shared" si="1"/>
-        <v>feveriosis_surveillance_zzz_2025_linelist_2_1</v>
+        <v>feveriosis_surveillance_zzz_2025_linelist_2_2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
[epirh] Adding example folder datasets
</commit_message>
<xml_diff>
--- a/inst/extdata/tableoftables.xlsx
+++ b/inst/extdata/tableoftables.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/luisfernandoquezada/Documents/GitHub/appliedepidata/inst/extdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2164287B-C64B-EF49-9B73-E6289DF431EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA4F97E1-17D5-1747-8E8E-1FDC2B07A506}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="19700" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1053" uniqueCount="281">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1193" uniqueCount="317">
   <si>
     <t>name</t>
   </si>
@@ -863,6 +863,114 @@
   </si>
   <si>
     <t>case_linelists_outbreak_sle_2014_dictionary_1_1</t>
+  </si>
+  <si>
+    <t>example_case_linelist_2020_10_08</t>
+  </si>
+  <si>
+    <t>example_case_linelist</t>
+  </si>
+  <si>
+    <t>Dated snapshot (2020-10-08) of fictional case linelist data for the West African Ebola outbreak of 2014, for an iteration/loops example folder (same content as linelist_raw)</t>
+  </si>
+  <si>
+    <t>example_case_linelist_outbreak_sle_2014</t>
+  </si>
+  <si>
+    <t>example_case_linelist_outbreak_sle_2014_linelist_1_1</t>
+  </si>
+  <si>
+    <t>example_hospital_linelists</t>
+  </si>
+  <si>
+    <t>Combined all-hospital cleaned linelist for the West African Ebola outbreak of 2014, for an iteration/loops example folder (same content as hospital_linelists)</t>
+  </si>
+  <si>
+    <t>example_case_linelist_outbreak_sle_2014_linelist_1_2</t>
+  </si>
+  <si>
+    <t>example_central_hospital</t>
+  </si>
+  <si>
+    <t>Central Hospital subset of the cleaned Ebola linelist, one of six per-hospital files for an iteration/loops example</t>
+  </si>
+  <si>
+    <t>example_case_linelist_outbreak_sle_2014_linelist_1_3</t>
+  </si>
+  <si>
+    <t>example_military_hospital</t>
+  </si>
+  <si>
+    <t>Military Hospital subset of the cleaned Ebola linelist, one of six per-hospital files for an iteration/loops example</t>
+  </si>
+  <si>
+    <t>example_case_linelist_outbreak_sle_2014_linelist_1_4</t>
+  </si>
+  <si>
+    <t>example_port_hospital</t>
+  </si>
+  <si>
+    <t>Port Hospital subset of the cleaned Ebola linelist, one of six per-hospital files for an iteration/loops example</t>
+  </si>
+  <si>
+    <t>example_case_linelist_outbreak_sle_2014_linelist_1_5</t>
+  </si>
+  <si>
+    <t>example_st_marks_maternity_hospital</t>
+  </si>
+  <si>
+    <t>St. Mark's Maternity Hospital (SMMH) subset of the cleaned Ebola linelist, one of six per-hospital files for an iteration/loops example</t>
+  </si>
+  <si>
+    <t>example_case_linelist_outbreak_sle_2014_linelist_1_6</t>
+  </si>
+  <si>
+    <t>example_missing</t>
+  </si>
+  <si>
+    <t>Missing-hospital subset of the cleaned Ebola linelist, one of six per-hospital files for an iteration/loops example</t>
+  </si>
+  <si>
+    <t>example_case_linelist_outbreak_sle_2014_linelist_1_7</t>
+  </si>
+  <si>
+    <t>example_other</t>
+  </si>
+  <si>
+    <t>Other-hospital subset of the cleaned Ebola linelist, one of six per-hospital files for an iteration/loops example</t>
+  </si>
+  <si>
+    <t>example_case_linelist_outbreak_sle_2014_linelist_1_8</t>
+  </si>
+  <si>
+    <t>example_fluH7N9_China_2013</t>
+  </si>
+  <si>
+    <t>example_influenza</t>
+  </si>
+  <si>
+    <t>Linelist data from an outbreak of influenza A H7N9 in China 2013, for an iteration/loops example folder (same content as fluH7N9_China_2013)</t>
+  </si>
+  <si>
+    <t>example_influenza_outbreak_chn_2013</t>
+  </si>
+  <si>
+    <t>example_influenza_outbreak_chn_2013_linelist_1_1</t>
+  </si>
+  <si>
+    <t>example_district_weekly_count_data</t>
+  </si>
+  <si>
+    <t>example_malaria</t>
+  </si>
+  <si>
+    <t>Fictional counts of malaria cases from Mozambique, for an iteration/loops example folder (same content as district_weekly_count_data)</t>
+  </si>
+  <si>
+    <t>example_malaria_outbreak_moz_2019</t>
+  </si>
+  <si>
+    <t>example_malaria_outbreak_moz_2019_aggregate_1_1</t>
   </si>
 </sst>
 </file>
@@ -1215,7 +1323,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Q75"/>
+  <dimension ref="A1:Q85"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="33" bestFit="1" customWidth="1"/>
@@ -1229,7 +1337,7 @@
     <col min="10" max="10" width="10.1640625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="7.5" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="5.1640625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="123" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="132.1640625" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="20.6640625" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="13.1640625" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="35.83203125" bestFit="1" customWidth="1"/>
@@ -5209,6 +5317,536 @@
       </c>
       <c r="Q75" t="s">
         <v>280</v>
+      </c>
+    </row>
+    <row r="76" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A76" t="s">
+        <v>281</v>
+      </c>
+      <c r="B76" t="s">
+        <v>18</v>
+      </c>
+      <c r="C76" t="s">
+        <v>19</v>
+      </c>
+      <c r="D76">
+        <v>1</v>
+      </c>
+      <c r="E76">
+        <v>1</v>
+      </c>
+      <c r="F76" t="s">
+        <v>20</v>
+      </c>
+      <c r="G76" t="s">
+        <v>101</v>
+      </c>
+      <c r="H76" t="s">
+        <v>93</v>
+      </c>
+      <c r="I76" t="s">
+        <v>282</v>
+      </c>
+      <c r="J76" t="s">
+        <v>24</v>
+      </c>
+      <c r="K76" t="s">
+        <v>47</v>
+      </c>
+      <c r="L76">
+        <v>2014</v>
+      </c>
+      <c r="M76" t="s">
+        <v>283</v>
+      </c>
+      <c r="N76" t="s">
+        <v>96</v>
+      </c>
+      <c r="O76" t="s">
+        <v>97</v>
+      </c>
+      <c r="P76" t="s">
+        <v>284</v>
+      </c>
+      <c r="Q76" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="77" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A77" t="s">
+        <v>286</v>
+      </c>
+      <c r="B77" t="s">
+        <v>18</v>
+      </c>
+      <c r="C77" t="s">
+        <v>19</v>
+      </c>
+      <c r="D77">
+        <v>1</v>
+      </c>
+      <c r="E77">
+        <v>2</v>
+      </c>
+      <c r="F77" t="s">
+        <v>20</v>
+      </c>
+      <c r="G77" t="s">
+        <v>101</v>
+      </c>
+      <c r="H77" t="s">
+        <v>93</v>
+      </c>
+      <c r="I77" t="s">
+        <v>282</v>
+      </c>
+      <c r="J77" t="s">
+        <v>24</v>
+      </c>
+      <c r="K77" t="s">
+        <v>47</v>
+      </c>
+      <c r="L77">
+        <v>2014</v>
+      </c>
+      <c r="M77" t="s">
+        <v>287</v>
+      </c>
+      <c r="N77" t="s">
+        <v>96</v>
+      </c>
+      <c r="O77" t="s">
+        <v>97</v>
+      </c>
+      <c r="P77" t="s">
+        <v>284</v>
+      </c>
+      <c r="Q77" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="78" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A78" t="s">
+        <v>289</v>
+      </c>
+      <c r="B78" t="s">
+        <v>18</v>
+      </c>
+      <c r="C78" t="s">
+        <v>82</v>
+      </c>
+      <c r="D78">
+        <v>1</v>
+      </c>
+      <c r="E78">
+        <v>3</v>
+      </c>
+      <c r="F78" t="s">
+        <v>20</v>
+      </c>
+      <c r="G78" t="s">
+        <v>101</v>
+      </c>
+      <c r="H78" t="s">
+        <v>93</v>
+      </c>
+      <c r="I78" t="s">
+        <v>282</v>
+      </c>
+      <c r="J78" t="s">
+        <v>24</v>
+      </c>
+      <c r="K78" t="s">
+        <v>47</v>
+      </c>
+      <c r="L78">
+        <v>2014</v>
+      </c>
+      <c r="M78" t="s">
+        <v>290</v>
+      </c>
+      <c r="N78" t="s">
+        <v>96</v>
+      </c>
+      <c r="O78" t="s">
+        <v>97</v>
+      </c>
+      <c r="P78" t="s">
+        <v>284</v>
+      </c>
+      <c r="Q78" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="79" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A79" t="s">
+        <v>292</v>
+      </c>
+      <c r="B79" t="s">
+        <v>18</v>
+      </c>
+      <c r="C79" t="s">
+        <v>82</v>
+      </c>
+      <c r="D79">
+        <v>1</v>
+      </c>
+      <c r="E79">
+        <v>4</v>
+      </c>
+      <c r="F79" t="s">
+        <v>20</v>
+      </c>
+      <c r="G79" t="s">
+        <v>101</v>
+      </c>
+      <c r="H79" t="s">
+        <v>93</v>
+      </c>
+      <c r="I79" t="s">
+        <v>282</v>
+      </c>
+      <c r="J79" t="s">
+        <v>24</v>
+      </c>
+      <c r="K79" t="s">
+        <v>47</v>
+      </c>
+      <c r="L79">
+        <v>2014</v>
+      </c>
+      <c r="M79" t="s">
+        <v>293</v>
+      </c>
+      <c r="N79" t="s">
+        <v>96</v>
+      </c>
+      <c r="O79" t="s">
+        <v>97</v>
+      </c>
+      <c r="P79" t="s">
+        <v>284</v>
+      </c>
+      <c r="Q79" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="80" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A80" t="s">
+        <v>295</v>
+      </c>
+      <c r="B80" t="s">
+        <v>18</v>
+      </c>
+      <c r="C80" t="s">
+        <v>82</v>
+      </c>
+      <c r="D80">
+        <v>1</v>
+      </c>
+      <c r="E80">
+        <v>5</v>
+      </c>
+      <c r="F80" t="s">
+        <v>20</v>
+      </c>
+      <c r="G80" t="s">
+        <v>101</v>
+      </c>
+      <c r="H80" t="s">
+        <v>93</v>
+      </c>
+      <c r="I80" t="s">
+        <v>282</v>
+      </c>
+      <c r="J80" t="s">
+        <v>24</v>
+      </c>
+      <c r="K80" t="s">
+        <v>47</v>
+      </c>
+      <c r="L80">
+        <v>2014</v>
+      </c>
+      <c r="M80" t="s">
+        <v>296</v>
+      </c>
+      <c r="N80" t="s">
+        <v>96</v>
+      </c>
+      <c r="O80" t="s">
+        <v>97</v>
+      </c>
+      <c r="P80" t="s">
+        <v>284</v>
+      </c>
+      <c r="Q80" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="81" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A81" t="s">
+        <v>298</v>
+      </c>
+      <c r="B81" t="s">
+        <v>18</v>
+      </c>
+      <c r="C81" t="s">
+        <v>82</v>
+      </c>
+      <c r="D81">
+        <v>1</v>
+      </c>
+      <c r="E81">
+        <v>6</v>
+      </c>
+      <c r="F81" t="s">
+        <v>20</v>
+      </c>
+      <c r="G81" t="s">
+        <v>101</v>
+      </c>
+      <c r="H81" t="s">
+        <v>93</v>
+      </c>
+      <c r="I81" t="s">
+        <v>282</v>
+      </c>
+      <c r="J81" t="s">
+        <v>24</v>
+      </c>
+      <c r="K81" t="s">
+        <v>47</v>
+      </c>
+      <c r="L81">
+        <v>2014</v>
+      </c>
+      <c r="M81" t="s">
+        <v>299</v>
+      </c>
+      <c r="N81" t="s">
+        <v>96</v>
+      </c>
+      <c r="O81" t="s">
+        <v>97</v>
+      </c>
+      <c r="P81" t="s">
+        <v>284</v>
+      </c>
+      <c r="Q81" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="82" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A82" t="s">
+        <v>301</v>
+      </c>
+      <c r="B82" t="s">
+        <v>18</v>
+      </c>
+      <c r="C82" t="s">
+        <v>82</v>
+      </c>
+      <c r="D82">
+        <v>1</v>
+      </c>
+      <c r="E82">
+        <v>7</v>
+      </c>
+      <c r="F82" t="s">
+        <v>20</v>
+      </c>
+      <c r="G82" t="s">
+        <v>101</v>
+      </c>
+      <c r="H82" t="s">
+        <v>93</v>
+      </c>
+      <c r="I82" t="s">
+        <v>282</v>
+      </c>
+      <c r="J82" t="s">
+        <v>24</v>
+      </c>
+      <c r="K82" t="s">
+        <v>47</v>
+      </c>
+      <c r="L82">
+        <v>2014</v>
+      </c>
+      <c r="M82" t="s">
+        <v>302</v>
+      </c>
+      <c r="N82" t="s">
+        <v>96</v>
+      </c>
+      <c r="O82" t="s">
+        <v>97</v>
+      </c>
+      <c r="P82" t="s">
+        <v>284</v>
+      </c>
+      <c r="Q82" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="83" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A83" t="s">
+        <v>304</v>
+      </c>
+      <c r="B83" t="s">
+        <v>18</v>
+      </c>
+      <c r="C83" t="s">
+        <v>82</v>
+      </c>
+      <c r="D83">
+        <v>1</v>
+      </c>
+      <c r="E83">
+        <v>8</v>
+      </c>
+      <c r="F83" t="s">
+        <v>20</v>
+      </c>
+      <c r="G83" t="s">
+        <v>101</v>
+      </c>
+      <c r="H83" t="s">
+        <v>93</v>
+      </c>
+      <c r="I83" t="s">
+        <v>282</v>
+      </c>
+      <c r="J83" t="s">
+        <v>24</v>
+      </c>
+      <c r="K83" t="s">
+        <v>47</v>
+      </c>
+      <c r="L83">
+        <v>2014</v>
+      </c>
+      <c r="M83" t="s">
+        <v>305</v>
+      </c>
+      <c r="N83" t="s">
+        <v>96</v>
+      </c>
+      <c r="O83" t="s">
+        <v>97</v>
+      </c>
+      <c r="P83" t="s">
+        <v>284</v>
+      </c>
+      <c r="Q83" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="84" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A84" t="s">
+        <v>307</v>
+      </c>
+      <c r="B84" t="s">
+        <v>18</v>
+      </c>
+      <c r="C84" t="s">
+        <v>82</v>
+      </c>
+      <c r="D84">
+        <v>1</v>
+      </c>
+      <c r="E84">
+        <v>1</v>
+      </c>
+      <c r="F84" t="s">
+        <v>20</v>
+      </c>
+      <c r="G84" t="s">
+        <v>92</v>
+      </c>
+      <c r="H84" t="s">
+        <v>93</v>
+      </c>
+      <c r="I84" t="s">
+        <v>308</v>
+      </c>
+      <c r="J84" t="s">
+        <v>24</v>
+      </c>
+      <c r="K84" t="s">
+        <v>25</v>
+      </c>
+      <c r="L84">
+        <v>2013</v>
+      </c>
+      <c r="M84" t="s">
+        <v>309</v>
+      </c>
+      <c r="N84" t="s">
+        <v>96</v>
+      </c>
+      <c r="O84" t="s">
+        <v>97</v>
+      </c>
+      <c r="P84" t="s">
+        <v>310</v>
+      </c>
+      <c r="Q84" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="85" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A85" t="s">
+        <v>312</v>
+      </c>
+      <c r="B85" t="s">
+        <v>81</v>
+      </c>
+      <c r="C85" t="s">
+        <v>19</v>
+      </c>
+      <c r="D85">
+        <v>1</v>
+      </c>
+      <c r="E85">
+        <v>1</v>
+      </c>
+      <c r="F85" t="s">
+        <v>20</v>
+      </c>
+      <c r="G85" t="s">
+        <v>152</v>
+      </c>
+      <c r="H85" t="s">
+        <v>22</v>
+      </c>
+      <c r="I85" t="s">
+        <v>313</v>
+      </c>
+      <c r="J85" t="s">
+        <v>24</v>
+      </c>
+      <c r="K85" t="s">
+        <v>47</v>
+      </c>
+      <c r="L85">
+        <v>2019</v>
+      </c>
+      <c r="M85" t="s">
+        <v>314</v>
+      </c>
+      <c r="N85" t="s">
+        <v>96</v>
+      </c>
+      <c r="O85" t="s">
+        <v>28</v>
+      </c>
+      <c r="P85" t="s">
+        <v>315</v>
+      </c>
+      <c r="Q85" t="s">
+        <v>316</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
[epirh] Adding gis_ datasets
</commit_message>
<xml_diff>
--- a/inst/extdata/tableoftables.xlsx
+++ b/inst/extdata/tableoftables.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/luisfernandoquezada/Documents/GitHub/appliedepidata/inst/extdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA4F97E1-17D5-1747-8E8E-1FDC2B07A506}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7A20780-7B04-CB40-B1B7-5BD8D4A0A739}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="19700" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1193" uniqueCount="317">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1249" uniqueCount="333">
   <si>
     <t>name</t>
   </si>
@@ -971,6 +971,54 @@
   </si>
   <si>
     <t>example_malaria_outbreak_moz_2019_aggregate_1_1</t>
+  </si>
+  <si>
+    <t>gis_population_sle_admpop_adm3_2020</t>
+  </si>
+  <si>
+    <t>gis_basics</t>
+  </si>
+  <si>
+    <t>mapping</t>
+  </si>
+  <si>
+    <t>Population data at admin level 3 for Sierra Leone from Humanitarian Data Exchange, repackaged for the GIS basics mapping example (same content as sle_admpop_adm3_2020)</t>
+  </si>
+  <si>
+    <t>gis_basics_sle_2020</t>
+  </si>
+  <si>
+    <t>gis_basics_sle_2020_population_1_1</t>
+  </si>
+  <si>
+    <t>gis_linelist_cleaned_with_adm3</t>
+  </si>
+  <si>
+    <t>Cleaned fictional Ebola Virus Disease linelist joined with admin-3 spatial data, repackaged for the GIS basics mapping example (same content as linelist_cleaned_with_adm3)</t>
+  </si>
+  <si>
+    <t>gis_basics_sle_2020_linelist_1_2</t>
+  </si>
+  <si>
+    <t>gis_covid_incidence</t>
+  </si>
+  <si>
+    <t>global</t>
+  </si>
+  <si>
+    <t>Fictional cumulative COVID-19 incidence by country, created for the GIS basics choropleth mapping example</t>
+  </si>
+  <si>
+    <t>gis_basics_sle_2020_aggregate_1_3</t>
+  </si>
+  <si>
+    <t>gis_population_sle_population_statistics_sierraleone_2020</t>
+  </si>
+  <si>
+    <t>Age/sex population proportions for Sierra Leone from Humanitarian Data Exchange, for the GIS basics population pyramid example</t>
+  </si>
+  <si>
+    <t>gis_basics_sle_2020_population_1_4</t>
   </si>
 </sst>
 </file>
@@ -1323,10 +1371,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Q85"/>
+  <dimension ref="A1:Q89"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="33" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="47.33203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="9.6640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11.1640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="11" bestFit="1" customWidth="1"/>
@@ -1337,7 +1385,7 @@
     <col min="10" max="10" width="10.1640625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="7.5" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="5.1640625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="132.1640625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="136.33203125" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="20.6640625" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="13.1640625" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="35.83203125" bestFit="1" customWidth="1"/>
@@ -5847,6 +5895,218 @@
       </c>
       <c r="Q85" t="s">
         <v>316</v>
+      </c>
+    </row>
+    <row r="86" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A86" t="s">
+        <v>317</v>
+      </c>
+      <c r="B86" t="s">
+        <v>32</v>
+      </c>
+      <c r="C86" t="s">
+        <v>82</v>
+      </c>
+      <c r="D86">
+        <v>1</v>
+      </c>
+      <c r="E86">
+        <v>1</v>
+      </c>
+      <c r="F86" t="s">
+        <v>20</v>
+      </c>
+      <c r="G86" t="s">
+        <v>101</v>
+      </c>
+      <c r="H86" t="s">
+        <v>93</v>
+      </c>
+      <c r="I86" t="s">
+        <v>318</v>
+      </c>
+      <c r="J86" t="s">
+        <v>319</v>
+      </c>
+      <c r="K86" t="s">
+        <v>25</v>
+      </c>
+      <c r="L86">
+        <v>2020</v>
+      </c>
+      <c r="M86" t="s">
+        <v>320</v>
+      </c>
+      <c r="N86" t="s">
+        <v>96</v>
+      </c>
+      <c r="O86" t="s">
+        <v>123</v>
+      </c>
+      <c r="P86" t="s">
+        <v>321</v>
+      </c>
+      <c r="Q86" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="87" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A87" t="s">
+        <v>323</v>
+      </c>
+      <c r="B87" t="s">
+        <v>18</v>
+      </c>
+      <c r="C87" t="s">
+        <v>67</v>
+      </c>
+      <c r="D87">
+        <v>1</v>
+      </c>
+      <c r="E87">
+        <v>2</v>
+      </c>
+      <c r="F87" t="s">
+        <v>20</v>
+      </c>
+      <c r="G87" t="s">
+        <v>101</v>
+      </c>
+      <c r="H87" t="s">
+        <v>93</v>
+      </c>
+      <c r="I87" t="s">
+        <v>318</v>
+      </c>
+      <c r="J87" t="s">
+        <v>319</v>
+      </c>
+      <c r="K87" t="s">
+        <v>47</v>
+      </c>
+      <c r="L87">
+        <v>2014</v>
+      </c>
+      <c r="M87" t="s">
+        <v>324</v>
+      </c>
+      <c r="N87" t="s">
+        <v>96</v>
+      </c>
+      <c r="O87" t="s">
+        <v>97</v>
+      </c>
+      <c r="P87" t="s">
+        <v>321</v>
+      </c>
+      <c r="Q87" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="88" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A88" t="s">
+        <v>326</v>
+      </c>
+      <c r="B88" t="s">
+        <v>81</v>
+      </c>
+      <c r="C88" t="s">
+        <v>82</v>
+      </c>
+      <c r="D88">
+        <v>1</v>
+      </c>
+      <c r="E88">
+        <v>3</v>
+      </c>
+      <c r="F88" t="s">
+        <v>20</v>
+      </c>
+      <c r="G88" t="s">
+        <v>327</v>
+      </c>
+      <c r="H88" t="s">
+        <v>327</v>
+      </c>
+      <c r="I88" t="s">
+        <v>318</v>
+      </c>
+      <c r="J88" t="s">
+        <v>319</v>
+      </c>
+      <c r="K88" t="s">
+        <v>47</v>
+      </c>
+      <c r="L88">
+        <v>2020</v>
+      </c>
+      <c r="M88" t="s">
+        <v>328</v>
+      </c>
+      <c r="N88" t="s">
+        <v>96</v>
+      </c>
+      <c r="O88" t="s">
+        <v>28</v>
+      </c>
+      <c r="P88" t="s">
+        <v>321</v>
+      </c>
+      <c r="Q88" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="89" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A89" t="s">
+        <v>330</v>
+      </c>
+      <c r="B89" t="s">
+        <v>32</v>
+      </c>
+      <c r="C89" t="s">
+        <v>19</v>
+      </c>
+      <c r="D89">
+        <v>1</v>
+      </c>
+      <c r="E89">
+        <v>4</v>
+      </c>
+      <c r="F89" t="s">
+        <v>20</v>
+      </c>
+      <c r="G89" t="s">
+        <v>101</v>
+      </c>
+      <c r="H89" t="s">
+        <v>93</v>
+      </c>
+      <c r="I89" t="s">
+        <v>318</v>
+      </c>
+      <c r="J89" t="s">
+        <v>319</v>
+      </c>
+      <c r="K89" t="s">
+        <v>25</v>
+      </c>
+      <c r="L89">
+        <v>2020</v>
+      </c>
+      <c r="M89" t="s">
+        <v>331</v>
+      </c>
+      <c r="N89" t="s">
+        <v>96</v>
+      </c>
+      <c r="O89" t="s">
+        <v>123</v>
+      </c>
+      <c r="P89" t="s">
+        <v>321</v>
+      </c>
+      <c r="Q89" t="s">
+        <v>332</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
[epirh] Adding epidemic mod and gis datasets
+ bug fixing
+ updating pkgdown
+ updating news
</commit_message>
<xml_diff>
--- a/inst/extdata/tableoftables.xlsx
+++ b/inst/extdata/tableoftables.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/luisfernandoquezada/Documents/GitHub/appliedepidata/inst/extdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7A20780-7B04-CB40-B1B7-5BD8D4A0A739}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4957B8AB-0A16-6548-909B-EE5D4A200723}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="19700" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="19720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1249" uniqueCount="333">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1431" uniqueCount="378">
   <si>
     <t>name</t>
   </si>
@@ -1019,6 +1019,141 @@
   </si>
   <si>
     <t>gis_basics_sle_2020_population_1_4</t>
+  </si>
+  <si>
+    <t>gis_africa_countries</t>
+  </si>
+  <si>
+    <t>json</t>
+  </si>
+  <si>
+    <t>afr</t>
+  </si>
+  <si>
+    <t>international</t>
+  </si>
+  <si>
+    <t>Natural Earth Admin-0 country boundaries filtered to the African continent, for the GIS basics mapping example</t>
+  </si>
+  <si>
+    <t>Public Domain</t>
+  </si>
+  <si>
+    <t>gis_basics_afr_2020</t>
+  </si>
+  <si>
+    <t>gis_basics_afr_2020_shape_1_1</t>
+  </si>
+  <si>
+    <t>linelist_cleaned</t>
+  </si>
+  <si>
+    <t>Cleaned fictional Ebola Virus Disease data simulating properties from the West African Ebola outbreak of 2014, added under a plain name (same content as linelist_cleaned_excel)</t>
+  </si>
+  <si>
+    <t>ebola_outbreak_sle_2014_linelist_1_6</t>
+  </si>
+  <si>
+    <t>epidemic_models_epinow_res</t>
+  </si>
+  <si>
+    <t>Outputs from {epinow2}, for the epidemic models example (same content as epinow_res)</t>
+  </si>
+  <si>
+    <t>epidemic_models_sle_2014</t>
+  </si>
+  <si>
+    <t>epidemic_models_sle_2014_other_1_1</t>
+  </si>
+  <si>
+    <t>epidemic_models_epinow_res_small</t>
+  </si>
+  <si>
+    <t>Outputs from {epinow2} (small), for the epidemic models example (same content as epinow_res_small)</t>
+  </si>
+  <si>
+    <t>epidemic_models_sle_2014_other_2_1</t>
+  </si>
+  <si>
+    <t>epidemic_models_generation_time</t>
+  </si>
+  <si>
+    <t>Generation time distribution, for the epidemic models example (same content as generation_time)</t>
+  </si>
+  <si>
+    <t>epidemic_models_sle_2014_other_3_1</t>
+  </si>
+  <si>
+    <t>epidemic_models_incubation_period</t>
+  </si>
+  <si>
+    <t>Incubation period distribution, for the epidemic models example (same content as incubation_period)</t>
+  </si>
+  <si>
+    <t>epidemic_models_sle_2014_other_4_1</t>
+  </si>
+  <si>
+    <t>epidemic_models_estimate_samples</t>
+  </si>
+  <si>
+    <t>Posterior estimate samples unbundled from epinow_res$estimates$samples, for the epidemic models example</t>
+  </si>
+  <si>
+    <t>epidemic_models_sle_2014_other_5_1</t>
+  </si>
+  <si>
+    <t>epidemic_models_estimated_reported_cases_samples</t>
+  </si>
+  <si>
+    <t>Posterior estimated-reported-cases samples unbundled from epinow_res$estimated_reported_cases$samples, for the epidemic models example</t>
+  </si>
+  <si>
+    <t>epidemic_models_sle_2014_other_6_1</t>
+  </si>
+  <si>
+    <t>epidemic_models_latest_date</t>
+  </si>
+  <si>
+    <t>Latest observation date unbundled from epinow_res$estimates$observations, for the epidemic models example</t>
+  </si>
+  <si>
+    <t>epidemic_models_sle_2014_other_7_1</t>
+  </si>
+  <si>
+    <t>epidemic_models_reported_cases</t>
+  </si>
+  <si>
+    <t>Reported case counts unbundled from epinow_res$estimates$observations, for the epidemic models example</t>
+  </si>
+  <si>
+    <t>epidemic_models_sle_2014_other_8_1</t>
+  </si>
+  <si>
+    <t>epidemic_models_summarised_estimated_reported_cases</t>
+  </si>
+  <si>
+    <t>Summarised estimated reported cases unbundled from epinow_res$estimated_reported_cases$summarised, for the epidemic models example</t>
+  </si>
+  <si>
+    <t>epidemic_models_sle_2014_other_9_1</t>
+  </si>
+  <si>
+    <t>epidemic_models_summarised_estimates</t>
+  </si>
+  <si>
+    <t>Summarised estimates unbundled from epinow_res$estimates$summarised, for the epidemic models example</t>
+  </si>
+  <si>
+    <t>epidemic_models_sle_2014_other_10_1</t>
+  </si>
+  <si>
+    <t>epidemic_models_summary</t>
+  </si>
+  <si>
+    <t>Model run summary unbundled from epinow_res$summary, for the epidemic models example</t>
+  </si>
+  <si>
+    <t>epidemic_models_sle_2014_other_11_1</t>
   </si>
 </sst>
 </file>
@@ -1371,7 +1506,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Q89"/>
+  <dimension ref="A1:Q102"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="47.33203125" bestFit="1" customWidth="1"/>
@@ -1380,12 +1515,12 @@
     <col min="5" max="5" width="11" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="8" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="7.1640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.1640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.1640625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="20.1640625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="10.1640625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="7.5" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="5.1640625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="136.33203125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="137.33203125" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="20.6640625" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="13.1640625" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="35.83203125" bestFit="1" customWidth="1"/>
@@ -6107,6 +6242,695 @@
       </c>
       <c r="Q89" t="s">
         <v>332</v>
+      </c>
+    </row>
+    <row r="90" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A90" t="s">
+        <v>333</v>
+      </c>
+      <c r="B90" t="s">
+        <v>36</v>
+      </c>
+      <c r="C90" t="s">
+        <v>334</v>
+      </c>
+      <c r="D90">
+        <v>1</v>
+      </c>
+      <c r="E90">
+        <v>1</v>
+      </c>
+      <c r="F90" t="s">
+        <v>20</v>
+      </c>
+      <c r="G90" t="s">
+        <v>335</v>
+      </c>
+      <c r="H90" t="s">
+        <v>336</v>
+      </c>
+      <c r="I90" t="s">
+        <v>318</v>
+      </c>
+      <c r="J90" t="s">
+        <v>319</v>
+      </c>
+      <c r="K90" t="s">
+        <v>25</v>
+      </c>
+      <c r="L90">
+        <v>2020</v>
+      </c>
+      <c r="M90" t="s">
+        <v>337</v>
+      </c>
+      <c r="N90" t="s">
+        <v>96</v>
+      </c>
+      <c r="O90" t="s">
+        <v>338</v>
+      </c>
+      <c r="P90" t="s">
+        <v>339</v>
+      </c>
+      <c r="Q90" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="91" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A91" t="s">
+        <v>341</v>
+      </c>
+      <c r="B91" t="s">
+        <v>18</v>
+      </c>
+      <c r="C91" t="s">
+        <v>19</v>
+      </c>
+      <c r="D91">
+        <v>1</v>
+      </c>
+      <c r="E91">
+        <v>6</v>
+      </c>
+      <c r="F91" t="s">
+        <v>20</v>
+      </c>
+      <c r="G91" t="s">
+        <v>101</v>
+      </c>
+      <c r="H91" t="s">
+        <v>93</v>
+      </c>
+      <c r="I91" t="s">
+        <v>102</v>
+      </c>
+      <c r="J91" t="s">
+        <v>24</v>
+      </c>
+      <c r="K91" t="s">
+        <v>47</v>
+      </c>
+      <c r="L91">
+        <v>2014</v>
+      </c>
+      <c r="M91" t="s">
+        <v>342</v>
+      </c>
+      <c r="N91" t="s">
+        <v>96</v>
+      </c>
+      <c r="O91" t="s">
+        <v>97</v>
+      </c>
+      <c r="P91" t="s">
+        <v>104</v>
+      </c>
+      <c r="Q91" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="92" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A92" t="s">
+        <v>344</v>
+      </c>
+      <c r="B92" t="s">
+        <v>130</v>
+      </c>
+      <c r="C92" t="s">
+        <v>67</v>
+      </c>
+      <c r="D92">
+        <v>1</v>
+      </c>
+      <c r="E92">
+        <v>1</v>
+      </c>
+      <c r="F92" t="s">
+        <v>20</v>
+      </c>
+      <c r="G92" t="s">
+        <v>101</v>
+      </c>
+      <c r="H92" t="s">
+        <v>93</v>
+      </c>
+      <c r="I92" t="s">
+        <v>102</v>
+      </c>
+      <c r="J92" t="s">
+        <v>24</v>
+      </c>
+      <c r="K92" t="s">
+        <v>47</v>
+      </c>
+      <c r="L92">
+        <v>2014</v>
+      </c>
+      <c r="M92" t="s">
+        <v>345</v>
+      </c>
+      <c r="N92" t="s">
+        <v>96</v>
+      </c>
+      <c r="O92" t="s">
+        <v>97</v>
+      </c>
+      <c r="P92" t="s">
+        <v>346</v>
+      </c>
+      <c r="Q92" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="93" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A93" t="s">
+        <v>348</v>
+      </c>
+      <c r="B93" t="s">
+        <v>130</v>
+      </c>
+      <c r="C93" t="s">
+        <v>67</v>
+      </c>
+      <c r="D93">
+        <v>2</v>
+      </c>
+      <c r="E93">
+        <v>1</v>
+      </c>
+      <c r="F93" t="s">
+        <v>20</v>
+      </c>
+      <c r="G93" t="s">
+        <v>101</v>
+      </c>
+      <c r="H93" t="s">
+        <v>93</v>
+      </c>
+      <c r="I93" t="s">
+        <v>102</v>
+      </c>
+      <c r="J93" t="s">
+        <v>24</v>
+      </c>
+      <c r="K93" t="s">
+        <v>47</v>
+      </c>
+      <c r="L93">
+        <v>2014</v>
+      </c>
+      <c r="M93" t="s">
+        <v>349</v>
+      </c>
+      <c r="N93" t="s">
+        <v>96</v>
+      </c>
+      <c r="O93" t="s">
+        <v>97</v>
+      </c>
+      <c r="P93" t="s">
+        <v>346</v>
+      </c>
+      <c r="Q93" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="94" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A94" t="s">
+        <v>351</v>
+      </c>
+      <c r="B94" t="s">
+        <v>130</v>
+      </c>
+      <c r="C94" t="s">
+        <v>67</v>
+      </c>
+      <c r="D94">
+        <v>3</v>
+      </c>
+      <c r="E94">
+        <v>1</v>
+      </c>
+      <c r="F94" t="s">
+        <v>20</v>
+      </c>
+      <c r="G94" t="s">
+        <v>101</v>
+      </c>
+      <c r="H94" t="s">
+        <v>93</v>
+      </c>
+      <c r="I94" t="s">
+        <v>102</v>
+      </c>
+      <c r="J94" t="s">
+        <v>24</v>
+      </c>
+      <c r="K94" t="s">
+        <v>47</v>
+      </c>
+      <c r="L94">
+        <v>2014</v>
+      </c>
+      <c r="M94" t="s">
+        <v>352</v>
+      </c>
+      <c r="N94" t="s">
+        <v>96</v>
+      </c>
+      <c r="O94" t="s">
+        <v>97</v>
+      </c>
+      <c r="P94" t="s">
+        <v>346</v>
+      </c>
+      <c r="Q94" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="95" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A95" t="s">
+        <v>354</v>
+      </c>
+      <c r="B95" t="s">
+        <v>130</v>
+      </c>
+      <c r="C95" t="s">
+        <v>67</v>
+      </c>
+      <c r="D95">
+        <v>4</v>
+      </c>
+      <c r="E95">
+        <v>1</v>
+      </c>
+      <c r="F95" t="s">
+        <v>20</v>
+      </c>
+      <c r="G95" t="s">
+        <v>101</v>
+      </c>
+      <c r="H95" t="s">
+        <v>93</v>
+      </c>
+      <c r="I95" t="s">
+        <v>102</v>
+      </c>
+      <c r="J95" t="s">
+        <v>24</v>
+      </c>
+      <c r="K95" t="s">
+        <v>47</v>
+      </c>
+      <c r="L95">
+        <v>2014</v>
+      </c>
+      <c r="M95" t="s">
+        <v>355</v>
+      </c>
+      <c r="N95" t="s">
+        <v>96</v>
+      </c>
+      <c r="O95" t="s">
+        <v>97</v>
+      </c>
+      <c r="P95" t="s">
+        <v>346</v>
+      </c>
+      <c r="Q95" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="96" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A96" t="s">
+        <v>357</v>
+      </c>
+      <c r="B96" t="s">
+        <v>130</v>
+      </c>
+      <c r="C96" t="s">
+        <v>67</v>
+      </c>
+      <c r="D96">
+        <v>5</v>
+      </c>
+      <c r="E96">
+        <v>1</v>
+      </c>
+      <c r="F96" t="s">
+        <v>20</v>
+      </c>
+      <c r="G96" t="s">
+        <v>101</v>
+      </c>
+      <c r="H96" t="s">
+        <v>93</v>
+      </c>
+      <c r="I96" t="s">
+        <v>102</v>
+      </c>
+      <c r="J96" t="s">
+        <v>24</v>
+      </c>
+      <c r="K96" t="s">
+        <v>47</v>
+      </c>
+      <c r="L96">
+        <v>2014</v>
+      </c>
+      <c r="M96" t="s">
+        <v>358</v>
+      </c>
+      <c r="N96" t="s">
+        <v>96</v>
+      </c>
+      <c r="O96" t="s">
+        <v>97</v>
+      </c>
+      <c r="P96" t="s">
+        <v>346</v>
+      </c>
+      <c r="Q96" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="97" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A97" t="s">
+        <v>360</v>
+      </c>
+      <c r="B97" t="s">
+        <v>130</v>
+      </c>
+      <c r="C97" t="s">
+        <v>67</v>
+      </c>
+      <c r="D97">
+        <v>6</v>
+      </c>
+      <c r="E97">
+        <v>1</v>
+      </c>
+      <c r="F97" t="s">
+        <v>20</v>
+      </c>
+      <c r="G97" t="s">
+        <v>101</v>
+      </c>
+      <c r="H97" t="s">
+        <v>93</v>
+      </c>
+      <c r="I97" t="s">
+        <v>102</v>
+      </c>
+      <c r="J97" t="s">
+        <v>24</v>
+      </c>
+      <c r="K97" t="s">
+        <v>47</v>
+      </c>
+      <c r="L97">
+        <v>2014</v>
+      </c>
+      <c r="M97" t="s">
+        <v>361</v>
+      </c>
+      <c r="N97" t="s">
+        <v>96</v>
+      </c>
+      <c r="O97" t="s">
+        <v>97</v>
+      </c>
+      <c r="P97" t="s">
+        <v>346</v>
+      </c>
+      <c r="Q97" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="98" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A98" t="s">
+        <v>363</v>
+      </c>
+      <c r="B98" t="s">
+        <v>130</v>
+      </c>
+      <c r="C98" t="s">
+        <v>67</v>
+      </c>
+      <c r="D98">
+        <v>7</v>
+      </c>
+      <c r="E98">
+        <v>1</v>
+      </c>
+      <c r="F98" t="s">
+        <v>20</v>
+      </c>
+      <c r="G98" t="s">
+        <v>101</v>
+      </c>
+      <c r="H98" t="s">
+        <v>93</v>
+      </c>
+      <c r="I98" t="s">
+        <v>102</v>
+      </c>
+      <c r="J98" t="s">
+        <v>24</v>
+      </c>
+      <c r="K98" t="s">
+        <v>47</v>
+      </c>
+      <c r="L98">
+        <v>2014</v>
+      </c>
+      <c r="M98" t="s">
+        <v>364</v>
+      </c>
+      <c r="N98" t="s">
+        <v>96</v>
+      </c>
+      <c r="O98" t="s">
+        <v>97</v>
+      </c>
+      <c r="P98" t="s">
+        <v>346</v>
+      </c>
+      <c r="Q98" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="99" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A99" t="s">
+        <v>366</v>
+      </c>
+      <c r="B99" t="s">
+        <v>130</v>
+      </c>
+      <c r="C99" t="s">
+        <v>67</v>
+      </c>
+      <c r="D99">
+        <v>8</v>
+      </c>
+      <c r="E99">
+        <v>1</v>
+      </c>
+      <c r="F99" t="s">
+        <v>20</v>
+      </c>
+      <c r="G99" t="s">
+        <v>101</v>
+      </c>
+      <c r="H99" t="s">
+        <v>93</v>
+      </c>
+      <c r="I99" t="s">
+        <v>102</v>
+      </c>
+      <c r="J99" t="s">
+        <v>24</v>
+      </c>
+      <c r="K99" t="s">
+        <v>47</v>
+      </c>
+      <c r="L99">
+        <v>2014</v>
+      </c>
+      <c r="M99" t="s">
+        <v>367</v>
+      </c>
+      <c r="N99" t="s">
+        <v>96</v>
+      </c>
+      <c r="O99" t="s">
+        <v>97</v>
+      </c>
+      <c r="P99" t="s">
+        <v>346</v>
+      </c>
+      <c r="Q99" t="s">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="100" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A100" t="s">
+        <v>369</v>
+      </c>
+      <c r="B100" t="s">
+        <v>130</v>
+      </c>
+      <c r="C100" t="s">
+        <v>67</v>
+      </c>
+      <c r="D100">
+        <v>9</v>
+      </c>
+      <c r="E100">
+        <v>1</v>
+      </c>
+      <c r="F100" t="s">
+        <v>20</v>
+      </c>
+      <c r="G100" t="s">
+        <v>101</v>
+      </c>
+      <c r="H100" t="s">
+        <v>93</v>
+      </c>
+      <c r="I100" t="s">
+        <v>102</v>
+      </c>
+      <c r="J100" t="s">
+        <v>24</v>
+      </c>
+      <c r="K100" t="s">
+        <v>47</v>
+      </c>
+      <c r="L100">
+        <v>2014</v>
+      </c>
+      <c r="M100" t="s">
+        <v>370</v>
+      </c>
+      <c r="N100" t="s">
+        <v>96</v>
+      </c>
+      <c r="O100" t="s">
+        <v>97</v>
+      </c>
+      <c r="P100" t="s">
+        <v>346</v>
+      </c>
+      <c r="Q100" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="101" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A101" t="s">
+        <v>372</v>
+      </c>
+      <c r="B101" t="s">
+        <v>130</v>
+      </c>
+      <c r="C101" t="s">
+        <v>67</v>
+      </c>
+      <c r="D101">
+        <v>10</v>
+      </c>
+      <c r="E101">
+        <v>1</v>
+      </c>
+      <c r="F101" t="s">
+        <v>20</v>
+      </c>
+      <c r="G101" t="s">
+        <v>101</v>
+      </c>
+      <c r="H101" t="s">
+        <v>93</v>
+      </c>
+      <c r="I101" t="s">
+        <v>102</v>
+      </c>
+      <c r="J101" t="s">
+        <v>24</v>
+      </c>
+      <c r="K101" t="s">
+        <v>47</v>
+      </c>
+      <c r="L101">
+        <v>2014</v>
+      </c>
+      <c r="M101" t="s">
+        <v>373</v>
+      </c>
+      <c r="N101" t="s">
+        <v>96</v>
+      </c>
+      <c r="O101" t="s">
+        <v>97</v>
+      </c>
+      <c r="P101" t="s">
+        <v>346</v>
+      </c>
+      <c r="Q101" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="102" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A102" t="s">
+        <v>375</v>
+      </c>
+      <c r="B102" t="s">
+        <v>130</v>
+      </c>
+      <c r="C102" t="s">
+        <v>67</v>
+      </c>
+      <c r="D102">
+        <v>11</v>
+      </c>
+      <c r="E102">
+        <v>1</v>
+      </c>
+      <c r="F102" t="s">
+        <v>20</v>
+      </c>
+      <c r="G102" t="s">
+        <v>101</v>
+      </c>
+      <c r="H102" t="s">
+        <v>93</v>
+      </c>
+      <c r="I102" t="s">
+        <v>102</v>
+      </c>
+      <c r="J102" t="s">
+        <v>24</v>
+      </c>
+      <c r="K102" t="s">
+        <v>47</v>
+      </c>
+      <c r="L102">
+        <v>2014</v>
+      </c>
+      <c r="M102" t="s">
+        <v>376</v>
+      </c>
+      <c r="N102" t="s">
+        <v>96</v>
+      </c>
+      <c r="O102" t="s">
+        <v>97</v>
+      </c>
+      <c r="P102" t="s">
+        <v>346</v>
+      </c>
+      <c r="Q102" t="s">
+        <v>377</v>
       </c>
     </row>
   </sheetData>

</xml_diff>